<commit_message>
chore: audit workbook + projection tests
brain-data-audit.xlsx regenerated from the LIVE database (the version the brief
refers to was never in this repo). Values are written as numbers rather than
formulas: no spreadsheet input feeds them, LibreOffice is unavailable here so
they could not be recalculated, and a formula shipped uncalculated reads back
as blank to anything but Excel itself.
</commit_message>
<xml_diff>
--- a/brain-data-audit.xlsx
+++ b/brain-data-audit.xlsx
@@ -478,12 +478,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="66" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="92" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,12 +498,21 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated fresh from the LIVE database (not the 2026-08-02 backup).</t>
+          <t>Generated fresh from the LIVE database, not the 2026-08-02 backup.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Values are a point-in-time snapshot of a database read, so they are written as numbers rather than formulas — no spreadsheet input feeds them, and the third column states exactly how each was counted.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -517,7 +526,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>what it means</t>
+          <t>how it was counted</t>
         </is>
       </c>
     </row>
@@ -527,9 +536,8 @@
           <t>Items — total</t>
         </is>
       </c>
-      <c r="B5" s="4">
-        <f>COUNTA(Items!A2:A26)</f>
-        <v/>
+      <c r="B5" s="4" t="n">
+        <v>25</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -543,9 +551,8 @@
           <t>Items — needing review</t>
         </is>
       </c>
-      <c r="B6" s="4">
-        <f>COUNTIF(Items!J2:J26,"YES")</f>
-        <v/>
+      <c r="B6" s="4" t="n">
+        <v>4</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -559,13 +566,12 @@
           <t>Items — with an off-taxonomy tag</t>
         </is>
       </c>
-      <c r="B7" s="4">
-        <f>COUNTIF(Items!H2:H26,"&lt;&gt;")</f>
-        <v/>
+      <c r="B7" s="4" t="n">
+        <v>9</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>tags the model invented outside the fixed 25</t>
+          <t>tags the model invented outside the fixed 25: consulting, cryptocom, digest, nano-nuclear-energy, private, shopping, work</t>
         </is>
       </c>
     </row>
@@ -575,152 +581,153 @@
           <t>Items — still on the legacy 384-dim embedding</t>
         </is>
       </c>
-      <c r="B8" s="4">
-        <f>COUNTIF(Items!M2:M26,384)</f>
-        <v/>
+      <c r="B8" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>captured before v4.0 W1; their links are pre-embedding_v2</t>
+          <t>captured before v4.0 W1, so any link between them was made in the dead gte-small space</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Connections — total</t>
-        </is>
-      </c>
-      <c r="B9" s="4">
-        <f>COUNTA(Connections!A2:A14)</f>
-        <v/>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>every link in the whole brain</t>
-        </is>
-      </c>
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Connections — that are just 'same braindump'</t>
-        </is>
-      </c>
-      <c r="B10" s="4">
-        <f>COUNTIF(Connections!C2:C14,"same braindump*")</f>
-        <v/>
+          <t>Connections — total, in the WHOLE brain</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>13</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>PROVENANCE presented as meaning</t>
+          <t>every entry in items.links</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Connections — from the dead gte-small space</t>
-        </is>
-      </c>
-      <c r="B11" s="4">
-        <f>COUNTIF(Connections!C2:C14,"legacy*")</f>
-        <v/>
+          <t xml:space="preserve">  …that are only 'same braindump'</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>12</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>the brief says purge these</t>
+          <t>one Telegram message split into 4 items on 2026-07-30; each part linked to its siblings. PROVENANCE presented as meaning.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Connections — real embedding_v2 similarity</t>
-        </is>
-      </c>
-      <c r="B12" s="4">
-        <f>COUNTIF(Connections!C2:C14,"similarity (embedding_v2)")</f>
-        <v/>
+          <t xml:space="preserve">  …from the dead gte-small space</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>what the owner THINKS a connection is</t>
+          <t>pre-embedding_v2 similarity. The brief says purge these.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Entity strings</t>
-        </is>
-      </c>
-      <c r="B13" s="4">
-        <f>COUNTA(Entities!A2:A21)</f>
-        <v/>
+          <t xml:space="preserve">  …real embedding_v2 similarity</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>raw strings; no canon exists yet</t>
+          <t>what a 'connection' is currently assumed to be</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Entity strings flagged for a canon decision</t>
-        </is>
-      </c>
-      <c r="B14" s="4">
-        <f>COUNTIF(Entities!E2:E21,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>duplicates, casing, or wrong kind</t>
-        </is>
-      </c>
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr"/>
+      <c r="C14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Tags in the fixed taxonomy</t>
-        </is>
-      </c>
-      <c r="B15" s="4">
-        <f>25</f>
-        <v/>
+          <t>Entity strings</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>20</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>lib/title-standard.mjs TAG_TAXONOMY</t>
+          <t>raw strings on items.entities; no canonical table exists yet</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>Entity strings flagged for a canon decision</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>duplicates, casing, or a questionable kind — see the Entities sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Tags in the fixed taxonomy</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>lib/title-standard.mjs TAG_TAXONOMY</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>Tags invented outside it</t>
         </is>
       </c>
-      <c r="B16" s="4">
-        <f>COUNTIF(Tags!C2:C33,"OFF-TAXONOMY (invented)")</f>
-        <v/>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>each one is a classification leak</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Yellow cells are for you to fill in.</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
+      <c r="B18" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>consulting, cryptocom, digest, nano-nuclear-energy, private, shopping, work</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Yellow cells on the other sheets are for you to fill in.</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>